<commit_message>
telefono y celular al colaborador
</commit_message>
<xml_diff>
--- a/src/main/resources/templates/excel/formatoProgramacion.xlsx
+++ b/src/main/resources/templates/excel/formatoProgramacion.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="21901"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B3F484C-201A-4F4F-AE79-262AD51F1BD1}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{040C46CE-22AD-49D6-B074-084DF260B21D}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -83,26 +83,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -125,23 +111,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>274320</xdr:colOff>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>106680</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>737858</xdr:colOff>
-      <xdr:row>4</xdr:row>
-      <xdr:rowOff>88900</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>113018</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Imagen 2">
+        <xdr:cNvPr id="2" name="Imagen 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4C734262-1CCE-4BC2-9F8A-E8E537DA9025}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{625481E2-384B-4165-9B3A-E9978D30B456}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -163,8 +149,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="274320" y="0"/>
-          <a:ext cx="882638" cy="838200"/>
+          <a:off x="480060" y="0"/>
+          <a:ext cx="836918" cy="662940"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -449,46 +435,46 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:15" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="1"/>
-      <c r="O1" s="1"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
+      <c r="I1" s="3"/>
+      <c r="J1" s="3"/>
+      <c r="K1" s="3"/>
+      <c r="L1" s="3"/>
+      <c r="M1" s="3"/>
+      <c r="N1" s="3"/>
+      <c r="O1" s="3"/>
     </row>
     <row r="2" spans="1:15" ht="14.55" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="8"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="1"/>
-      <c r="O2" s="1"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+      <c r="H2" s="3"/>
+      <c r="I2" s="3"/>
+      <c r="J2" s="3"/>
+      <c r="K2" s="3"/>
+      <c r="L2" s="3"/>
+      <c r="M2" s="3"/>
+      <c r="N2" s="3"/>
+      <c r="O2" s="3"/>
     </row>
-    <row r="3" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" s="8"/>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
+    <row r="3" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -498,40 +484,37 @@
       <c r="K3" s="3"/>
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
-      <c r="N3" s="1"/>
-      <c r="O3" s="1"/>
+      <c r="N3" s="3"/>
+      <c r="O3" s="3"/>
     </row>
-    <row r="4" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="9"/>
-      <c r="B4" s="9"/>
-      <c r="C4" s="9"/>
-      <c r="D4" s="9"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
-      <c r="I4" s="4"/>
-      <c r="J4" s="4"/>
-      <c r="K4" s="4"/>
-      <c r="L4" s="4"/>
-      <c r="M4" s="4"/>
-      <c r="N4" s="1"/>
-      <c r="O4" s="1"/>
+    <row r="4" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="3"/>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
+      <c r="J4" s="3"/>
+      <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
+      <c r="O4" s="3"/>
     </row>
-    <row r="5" spans="1:15" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="6" t="s">
+    <row r="5" spans="1:15" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="1"/>
+      <c r="B5" s="1"/>
+      <c r="C5" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="6"/>
+      <c r="D5" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="A4:D4"/>
+  <mergeCells count="1">
+    <mergeCell ref="A1:O4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="124" orientation="portrait" horizontalDpi="203" verticalDpi="203" r:id="rId1"/>

</xml_diff>